<commit_message>
update the agents dwh database and fix the email retrieval instead of cm to dwh
</commit_message>
<xml_diff>
--- a/app/CM/CM_Users.xlsx
+++ b/app/CM/CM_Users.xlsx
@@ -417,823 +417,3479 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:U47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>UniqueId</t>
+          <t>AccountID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>CreationDateTime</t>
+          <t>AccountCreationDateTime</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>EmailAddress</t>
+          <t>AccountEmailAddress</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>LastUpdatedDateTime</t>
+          <t>AccountLastUpdatedDateTime</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>PersonID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Avatar</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>PersonCreationDateTime</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Discriminator</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>PersonEmailAddress</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ExternalIdentifier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FirstName</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>LastName</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>FullName</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>PersonLastUpdatedDateTime</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>MaxChats</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>MaxWaitingChats</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>UserPresence</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>LastSentDateTime</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ContactGroup_UniqueId</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Account_UniqueID</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>UserEmailAddress</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FF06668B-F9AE-EF11-88CF-000D3A274416</t>
+          <t>3C98D1CB-84D3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45626.37535763889</v>
+        <v>45021.31820451389</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nada.Abdullah@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="n">
-        <v>45645.42101975694</v>
+          <t>Al_Andalusia_Group_CM_Admin@cmactivation.nl</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3D98D1CB-84D3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="1" t="n">
+        <v>45021.31820451389</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Al Andalusia Group</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al Andalusia Group </t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="n">
+        <v>46176.70494741898</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="n">
+        <v>46105.58050350694</v>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>3C98D1CB-84D3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Al_Andalusia_Group_CM_Admin@cmactivation.nl</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1004FCDC-4786-EF11-8473-000D3AAA2145</t>
+          <t>1721E9A5-8AD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45574.58881631945</v>
+        <v>45021.34727523148</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hassan-mohammed@andalusiagroup.net</t>
+          <t>Karim.AbuAuf@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>45832.47076015046</v>
+        <v>45550.31502635417</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1921E9A5-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="1" t="n">
+        <v>45021.34727523148</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sara</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>AbdElShafi</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Sara AbdElShafi</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>46218.7241221412</v>
+      </c>
+      <c r="O3" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="n">
+        <v>46218.58939186342</v>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>1721E9A5-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Sara.AbdElShafi@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6686991F-A775-EE11-8923-000D3AACCC78</t>
+          <t>F2DBD0C3-8AD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45227.64728144676</v>
+        <v>45021.34785072917</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>emad.shokry@andalusiagroup.net</t>
+          <t>Rania-Mohamed@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D4" s="1" t="n">
-        <v>45792.38513584491</v>
+        <v>45574.22003515047</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>F3DBD0C3-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="1" t="n">
+        <v>45021.34785072917</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Ibrahim</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Awad</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Ibrahim Awad</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>46217.86514560185</v>
+      </c>
+      <c r="O4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>46217.83056443287</v>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>F2DBD0C3-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Ibrahim-Qarni@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7566B5A5-C975-EE11-8923-000D3AACCC78</t>
+          <t>4031B6E1-8AD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>45227.81878873843</v>
+        <v>45021.34841759259</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nagham-katamish@andalusiagroup.net</t>
+          <t>Dina-Fathy@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D5" s="1" t="n">
-        <v>45589.20556091435</v>
-      </c>
+        <v>45288.52562190972</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4131B6E1-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="1" t="n">
+        <v>45021.34841759259</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>fathy</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Dina fathy</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="n">
+        <v>45288.52562190972</v>
+      </c>
+      <c r="O5" t="n">
+        <v>100</v>
+      </c>
+      <c r="P5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R5" s="1" t="n">
+        <v>45288.30898688657</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>4031B6E1-8AD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3FD1188C-817C-EE11-8923-000D3AACCC78</t>
+          <t>EE938441-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>45236.36845876157</v>
+        <v>45021.35022728009</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yosra.Hamed@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Salma.Abdelrahman@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>45648.30281616898</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EF938441-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="1" t="n">
+        <v>45021.35022728009</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>salma</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Abdelrahman</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>salma Abdelrahman</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="n">
+        <v>46219.02665697916</v>
+      </c>
+      <c r="O6" t="n">
+        <v>100</v>
+      </c>
+      <c r="P6" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R6" s="1" t="n">
+        <v>46218.73200104167</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>EE938441-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Salma.Abdelrahman@Andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5470C2D5-7B51-EF11-86C3-00224882330F</t>
+          <t>CC8E6465-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>45507.40024019676</v>
+        <v>45021.35095408565</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Esraa.Yousef@Andalusiagroup.net</t>
+          <t>Dalal.Gouda@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>45690.55735008102</v>
-      </c>
+        <v>45288.54031501157</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CD8E6465-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="1" t="n">
+        <v>45021.35095408565</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Dalal</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Gouda</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Dalal Gouda</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>45288.54031501157</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="n">
+        <v>45287.29972549769</v>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>CC8E6465-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3C98D1CB-84D3-ED11-9F74-6045BD88224D</t>
+          <t>8F355883-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>45021.31820451389</v>
+        <v>45021.35160061342</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Al_Andalusia_Group_CM_Admin@cmactivation.nl</t>
+          <t>Youstina.Malak@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>90355883-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="1" t="n">
+        <v>45021.35160061342</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yostina </t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>malak</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>yostina  malak</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>46218.90704394676</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R8" s="1" t="n">
+        <v>46073.31136230324</v>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>8F355883-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Youstina.Malak@Andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1721E9A5-8AD3-ED11-9F74-6045BD88224D</t>
+          <t>5B4D5EA7-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>45021.34727523148</v>
+        <v>45021.35225008102</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Karim.AbuAuf@Andalusiagroup.net</t>
+          <t>Lugien.AboElSoud@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>45550.31502635417</v>
-      </c>
+        <v>45266.72402815972</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5D4D5EA7-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="1" t="n">
+        <v>45021.35225008102</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lugien </t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>mohammed</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>lugien  mohammed</t>
+        </is>
+      </c>
+      <c r="N9" s="1" t="n">
+        <v>45266.72402815972</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R9" s="1" t="n">
+        <v>45048.43064626157</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>5B4D5EA7-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F2DBD0C3-8AD3-ED11-9F74-6045BD88224D</t>
+          <t>BE2C44BF-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>45021.34785072917</v>
+        <v>45021.35275162037</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rania-Mohamed@andalusiagroup.net</t>
+          <t>AbdElAziz.Kamal@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>45574.22003515047</v>
-      </c>
+        <v>45154.46350373843</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>C02C44BF-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="1" t="n">
+        <v>45021.35275162037</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdelaziz  </t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kamal </t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdelaziz   Kamal </t>
+        </is>
+      </c>
+      <c r="N10" s="1" t="n">
+        <v>45154.46350373843</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R10" s="1" t="n">
+        <v>45059.42744282408</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BE2C44BF-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4031B6E1-8AD3-ED11-9F74-6045BD88224D</t>
+          <t>59DA2BDD-8BD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>45021.34841759259</v>
+        <v>45021.35332126157</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dina-Fathy@Andalusiagroup.net</t>
+          <t>Abdelaziz.elnaggar@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>45288.52562190972</v>
-      </c>
+        <v>45288.54607361111</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>5ADA2BDD-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="1" t="n">
+        <v>45021.35332126157</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abdelaziz </t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Elnaggar</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Abdelaziz  Elnaggar</t>
+        </is>
+      </c>
+      <c r="N11" s="1" t="n">
+        <v>45288.54607361111</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R11" s="1" t="n">
+        <v>45286.74247063657</v>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>59DA2BDD-8BD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EE938441-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>1F3E94E4-8CD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>45021.35022728009</v>
+        <v>45021.35842384259</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Salma.Abdelrahman@Andalusiagroup.net</t>
+          <t>Omar.Shehata@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>45648.30281616898</v>
+        <v>45605.02578692129</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>203E94E4-8CD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="1" t="n">
+        <v>45021.35842384259</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Omar </t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Shehata</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Omar  Shehata</t>
+        </is>
+      </c>
+      <c r="N12" s="1" t="n">
+        <v>46218.98535582176</v>
+      </c>
+      <c r="O12" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R12" s="1" t="n">
+        <v>46218.87406334491</v>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1F3E94E4-8CD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Omar.Shehata@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CC8E6465-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>B5989508-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>45021.35095408565</v>
+        <v>45021.35911674768</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dalal.Gouda@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>45288.54031501157</v>
+          <t>Dalia.Abdellatif@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B6989508-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" s="1" t="n">
+        <v>45021.35911674768</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Kerolos</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Mories</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Kerolos Mories</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="n">
+        <v>46218.83344394676</v>
+      </c>
+      <c r="O13" t="n">
+        <v>10</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R13" s="1" t="n">
+        <v>46218.81586420139</v>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>B5989508-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Kerolos.Mories@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8F355883-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>B16C7732-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>45021.35160061342</v>
+        <v>45021.35990466435</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Youstina.Malak@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>Eman-Abdrabo@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>45494.35123611111</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B26C7732-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" s="1" t="n">
+        <v>45021.35990466435</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eman </t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Abdrabo</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Eman  Abdrabo</t>
+        </is>
+      </c>
+      <c r="N14" s="1" t="n">
+        <v>45494.35123611111</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R14" s="1" t="n">
+        <v>45039.55688741898</v>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>B16C7732-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5B4D5EA7-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>B336686E-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>45021.35225008102</v>
+        <v>45021.36110471065</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lugien.AboElSoud@Andalusiagroup.net</t>
+          <t>Mohamed.ElYamani@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>45266.72402815972</v>
+        <v>45702.62967137731</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>B436686E-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" s="1" t="n">
+        <v>45021.36110471065</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Kamal</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Mohamed Kamal</t>
+        </is>
+      </c>
+      <c r="N15" s="1" t="n">
+        <v>46217.88959189815</v>
+      </c>
+      <c r="O15" t="n">
+        <v>10</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R15" s="1" t="n">
+        <v>46217.87533684028</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>B336686E-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>kamal-elsayed@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BE2C44BF-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>15315DB0-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>45021.35275162037</v>
+        <v>45021.36232241898</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AbdElAziz.Kamal@Andalusiagroup.net</t>
+          <t>ERS-CC-TeamLeaders@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>45154.46350373843</v>
-      </c>
+        <v>45706.55016913194</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>16315DB0-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" s="1" t="n">
+        <v>45021.36232241898</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Amr</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Atef</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Amr Atef</t>
+        </is>
+      </c>
+      <c r="N16" s="1" t="n">
+        <v>45706.55028738426</v>
+      </c>
+      <c r="O16" t="n">
+        <v>110000</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>15315DB0-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>59DA2BDD-8BD3-ED11-9F74-6045BD88224D</t>
+          <t>04B540C8-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>45021.35332126157</v>
+        <v>45021.36280917824</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Abdelaziz.elnaggar@Andalusiagroup.net</t>
+          <t>ERS-CC-QualityManagement@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>45288.54607361111</v>
+        <v>45596.52452152778</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>05B540C8-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" s="1" t="n">
+        <v>45021.36280917824</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>46218.76559545139</v>
+      </c>
+      <c r="O17" t="n">
+        <v>100</v>
+      </c>
+      <c r="P17" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>04B540C8-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>ers-cc-qualitymanagement@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1F3E94E4-8CD3-ED11-9F74-6045BD88224D</t>
+          <t>5A0626E6-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>45021.35842384259</v>
+        <v>45021.36339795139</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Omar.Shehata@Andalusiagroup.net</t>
+          <t>Amal.Nabil@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>45605.02578692129</v>
-      </c>
+        <v>45494.35013475695</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5C0626E6-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" s="1" t="n">
+        <v>45021.36339795139</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amal </t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Nabil Mohamed Ahmed</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Amal  Nabil Mohamed Ahmed</t>
+        </is>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>45494.35013475695</v>
+      </c>
+      <c r="O18" t="n">
+        <v>100</v>
+      </c>
+      <c r="P18" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>5A0626E6-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B5989508-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>03D617FE-8DD3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>45021.35911674768</v>
+        <v>45021.36389082176</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dalia.Abdellatif@Andalusiagroup.net</t>
+          <t>Peter.Kamal@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>04D617FE-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" s="1" t="n">
+        <v>45021.36389082176</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peter </t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Magdy Kamal</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Peter  Magdy Kamal</t>
+        </is>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>46197.91318657407</v>
+      </c>
+      <c r="O19" t="n">
+        <v>100</v>
+      </c>
+      <c r="P19" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>03D617FE-8DD3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Peter.Kamal@Andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B16C7732-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>919F0916-8ED3-ED11-9F74-6045BD88224D</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>45021.35990466435</v>
+        <v>45021.36435431713</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eman-Abdrabo@Andalusiagroup.net</t>
+          <t>ERS-ITDigital@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>45494.35123611111</v>
+        <v>45742.3744619213</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>929F0916-8ED3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" s="1" t="n">
+        <v>45021.36435431713</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ERS-ITDigital</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>ERS-ITDigital</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>ERS-ITDigital ERS-ITDigital</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>46218.43004548611</v>
+      </c>
+      <c r="O20" t="n">
+        <v>100</v>
+      </c>
+      <c r="P20" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R20" s="1" t="n">
+        <v>45907.3964940162</v>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>919F0916-8ED3-ED11-9F74-6045BD88224D</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>ERS-ITDigital@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B336686E-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>F5894630-80A5-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>45021.36110471065</v>
+        <v>45288.53760663194</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mohamed.ElYamani@Andalusiagroup.net</t>
+          <t>Hager-AbdElGhany@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>45702.62967137731</v>
+        <v>45730.46219788194</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>F7894630-80A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" s="1" t="n">
+        <v>45288.53760663194</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Shaban</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Mohamed Shaban</t>
+        </is>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>46217.99418862269</v>
+      </c>
+      <c r="O21" t="n">
+        <v>10</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R21" s="1" t="n">
+        <v>46218.95444059028</v>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>F5894630-80A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Mohamed.Refaai@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>15315DB0-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>3AB179EA-80A5-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>45021.36232241898</v>
+        <v>45288.54126331019</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ERS-CC-TeamLeaders@Andalusiagroup.net</t>
+          <t>AbdelAal.Mohsen@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>45706.55016913194</v>
+        <v>45794.98535142361</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>3BB179EA-80A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" s="1" t="n">
+        <v>45288.54126331019</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Mariam</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Ossama</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Mariam Ossama</t>
+        </is>
+      </c>
+      <c r="N22" s="1" t="n">
+        <v>46218.63518306713</v>
+      </c>
+      <c r="O22" t="n">
+        <v>10</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R22" s="1" t="n">
+        <v>46218.63513078704</v>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>3AB179EA-80A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>mariam.galaleldin@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04B540C8-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>2611E2E6-81A5-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>45021.36280917824</v>
+        <v>45288.54612149305</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ERS-CC-QualityManagement@Andalusiagroup.net</t>
+          <t>Mohamed.ElYamani1@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>45596.52452152778</v>
-      </c>
+        <v>45525.34441952546</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2711E2E6-81A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" s="1" t="n">
+        <v>45288.54612149305</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Magdy ElYamani Ali</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Mohamed Magdy ElYamani Ali</t>
+        </is>
+      </c>
+      <c r="N23" s="1" t="n">
+        <v>45288.54629456018</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100</v>
+      </c>
+      <c r="P23" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2611E2E6-81A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5A0626E6-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>16050161-253C-EE11-B8F0-6045BD8BD59A</t>
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>45021.36339795139</v>
+        <v>45154.4650746875</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Amal.Nabil@Andalusiagroup.net</t>
+          <t>Ashraf.Abdullah@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>45494.35013475695</v>
-      </c>
+        <v>45202.58992144676</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>17050161-253C-EE11-B8F0-6045BD8BD59A</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" s="1" t="n">
+        <v>45154.4650746875</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>AbdElrahman</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>AbdElrahman Abdullah</t>
+        </is>
+      </c>
+      <c r="N24" s="1" t="n">
+        <v>45202.58992144676</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100</v>
+      </c>
+      <c r="P24" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="R24" s="1" t="n">
+        <v>45182.65361481482</v>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>16050161-253C-EE11-B8F0-6045BD8BD59A</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>03D617FE-8DD3-ED11-9F74-6045BD88224D</t>
+          <t>FF06668B-F9AE-EF11-88CF-000D3A274416</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>45021.36389082176</v>
+        <v>45626.37535763889</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Peter.Kamal@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>Nada.Abdullah@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>45645.42101975694</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>E506668B-F9AE-EF11-88CF-000D3A274416</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" s="1" t="n">
+        <v>45626.37535258102</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Nada</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Essam</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Nada Essam</t>
+        </is>
+      </c>
+      <c r="N25" s="1" t="n">
+        <v>46218.7371128125</v>
+      </c>
+      <c r="O25" t="n">
+        <v>10</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R25" s="1" t="n">
+        <v>46218.63074305555</v>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>FF06668B-F9AE-EF11-88CF-000D3A274416</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>nada.abdullah@andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>919F0916-8ED3-ED11-9F74-6045BD88224D</t>
+          <t>6686991F-A775-EE11-8923-000D3AACCC78</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>45021.36435431713</v>
+        <v>45227.64728144676</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ERS-ITDigital@Andalusiagroup.net</t>
+          <t>emad.shokry@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>45742.3744619213</v>
+        <v>45792.38513584491</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>6786991F-A775-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" s="1" t="n">
+        <v>45227.64728144676</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Farouk</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Youssef Farouk</t>
+        </is>
+      </c>
+      <c r="N26" s="1" t="n">
+        <v>46218.99893665509</v>
+      </c>
+      <c r="O26" t="n">
+        <v>10</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R26" s="1" t="n">
+        <v>46218.87118596065</v>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>6686991F-A775-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>youssef-farouk@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FE49D87E-8B2F-EE11-B8F0-6045BD8BD59A</t>
+          <t>7566B5A5-C975-EE11-8923-000D3AACCC78</t>
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>45138.4290727199</v>
+        <v>45227.81878873843</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mahmoud.Farghel@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>nagham-katamish@andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>45589.20556091435</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>7666B5A5-C975-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" s="1" t="n">
+        <v>45227.81878873843</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Ehab</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>AbdElMonem</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Ehab AbdElMonem</t>
+        </is>
+      </c>
+      <c r="N27" s="1" t="n">
+        <v>46218.8324227662</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R27" s="1" t="n">
+        <v>46218.83239869213</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>7566B5A5-C975-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>ehab.shehabeldin@andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16050161-253C-EE11-B8F0-6045BD8BD59A</t>
+          <t>CBCB121D-5394-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>45154.4650746875</v>
+        <v>45266.67968457176</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ashraf.Abdullah@Andalusiagroup.net</t>
+          <t>nagham-katamish1@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D28" s="1" t="n">
-        <v>45202.58992144676</v>
+        <v>45791.43502630787</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>CFCB121D-5394-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" s="1" t="n">
+        <v>45266.67968457176</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Hoda</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Moustafa</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Hoda Moustafa</t>
+        </is>
+      </c>
+      <c r="N28" s="1" t="n">
+        <v>46200.59510725694</v>
+      </c>
+      <c r="O28" t="n">
+        <v>10</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R28" s="1" t="n">
+        <v>46128.45420390047</v>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>CBCB121D-5394-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Hoda.Hassan@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>322B5412-FE29-EE11-A9BB-6045BD8BDAB6</t>
+          <t>A3E68C53-5C94-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>45131.36315601852</v>
+        <v>45266.72544401621</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mohanad.Zakaria@Andalusiagroup.net</t>
+          <t>emad.shokry1@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D29" s="1" t="n">
-        <v>45819.51390902778</v>
+        <v>45598.48289579861</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>A4E68C53-5C94-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" s="1" t="n">
+        <v>45266.72544401621</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AbdElRahman </t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> AlQadi</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>AbdElRahman   AlQadi</t>
+        </is>
+      </c>
+      <c r="N29" s="1" t="n">
+        <v>46217.86100239583</v>
+      </c>
+      <c r="O29" t="n">
+        <v>10</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R29" s="1" t="n">
+        <v>46217.8609909375</v>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>A3E68C53-5C94-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>AbdElRahman.AlQadi@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7FD59615-D2F7-ED11-907C-6045BD91ED88</t>
+          <t>5470C2D5-7B51-EF11-86C3-00224882330F</t>
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>45067.51534633102</v>
+        <v>45507.40024019676</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Montasser.Yahia@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>Esraa.Yousef@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>45690.55735008102</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>5570C2D5-7B51-EF11-86C3-00224882330F</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" s="1" t="n">
+        <v>45507.40024019676</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Esraa</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yousef </t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esraa Yousef </t>
+        </is>
+      </c>
+      <c r="N30" s="1" t="n">
+        <v>46218.70339552083</v>
+      </c>
+      <c r="O30" t="n">
+        <v>10</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R30" s="1" t="n">
+        <v>46218.53890258102</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>5470C2D5-7B51-EF11-86C3-00224882330F</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Esraa.Yousef@Andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CBCB121D-5394-EE11-8923-6045BD9E3927</t>
+          <t>322B5412-FE29-EE11-A9BB-6045BD8BDAB6</t>
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>45266.67968457176</v>
+        <v>45131.36315601852</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>nagham-katamish1@andalusiagroup.net</t>
+          <t>Mohanad.Zakaria@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D31" s="1" t="n">
-        <v>45791.43502630787</v>
+        <v>45819.51390902778</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>332B5412-FE29-EE11-A9BB-6045BD8BDAB6</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://robincontentdesktop.blob.core.windows.net/images/35033/avatars/332b5412-fe29-ee11-a9bb-6045bd8bdab6_40px.png</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="n">
+        <v>45131.36315601852</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Menna</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Fathy</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Menna Fathy</t>
+        </is>
+      </c>
+      <c r="N31" s="1" t="n">
+        <v>46200.56007700232</v>
+      </c>
+      <c r="O31" t="n">
+        <v>10</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R31" s="1" t="n">
+        <v>46188.49424247685</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>322B5412-FE29-EE11-A9BB-6045BD8BDAB6</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Mennatallah.Fathy@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>A3E68C53-5C94-EE11-8923-6045BD9E3927</t>
+          <t>7FD59615-D2F7-ED11-907C-6045BD91ED88</t>
         </is>
       </c>
       <c r="B32" s="1" t="n">
-        <v>45266.72544401621</v>
+        <v>45067.51534633102</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>emad.shokry1@andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>45598.48289579861</v>
-      </c>
+          <t>Montasser.Yahia@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>80D59615-D2F7-ED11-907C-6045BD91ED88</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" s="1" t="n">
+        <v>45067.51534633102</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Montasser</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Yahia</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Montasser Yahia</t>
+        </is>
+      </c>
+      <c r="N32" s="1" t="n">
+        <v>45927.4174681713</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>7FD59615-D2F7-ED11-907C-6045BD91ED88</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>F5894630-80A5-EE11-8923-6045BD9E3927</t>
+          <t>B278C7C1-D469-EF11-BDFD-6045BD9E3927</t>
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>45288.53760663194</v>
+        <v>45538.38429707176</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Hager-AbdElGhany@Andalusiagroup.net</t>
+          <t>Mona-Hassan@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D33" s="1" t="n">
-        <v>45730.46219788194</v>
+        <v>45801.51275</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>B478C7C1-D469-EF11-BDFD-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" s="1" t="n">
+        <v>45538.38429707176</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hager </t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mohamed </t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hager  Mohamed </t>
+        </is>
+      </c>
+      <c r="N33" s="1" t="n">
+        <v>46218.55577916667</v>
+      </c>
+      <c r="O33" t="n">
+        <v>10</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R33" s="1" t="n">
+        <v>46217.49769571759</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>B278C7C1-D469-EF11-BDFD-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Hager.Hanafy@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3AB179EA-80A5-EE11-8923-6045BD9E3927</t>
+          <t>1004FCDC-4786-EF11-8473-000D3AAA2145</t>
         </is>
       </c>
       <c r="B34" s="1" t="n">
-        <v>45288.54126331019</v>
+        <v>45574.58881631945</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AbdelAal.Mohsen@Andalusiagroup.net</t>
+          <t>Hassan-mohammed@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D34" s="1" t="n">
-        <v>45794.98535142361</v>
+        <v>45832.47076015046</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0E04FCDC-4786-EF11-8473-000D3AAA2145</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" s="1" t="n">
+        <v>45574.58881307871</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Nesma</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Youssef</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Nesma Youssef</t>
+        </is>
+      </c>
+      <c r="N34" s="1" t="n">
+        <v>46218.63265158565</v>
+      </c>
+      <c r="O34" t="n">
+        <v>10</v>
+      </c>
+      <c r="P34" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R34" s="1" t="n">
+        <v>46218.63247109954</v>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>1004FCDC-4786-EF11-8473-000D3AAA2145</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Nesma.Youssef@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2611E2E6-81A5-EE11-8923-6045BD9E3927</t>
+          <t>FE49D87E-8B2F-EE11-B8F0-6045BD8BD59A</t>
         </is>
       </c>
       <c r="B35" s="1" t="n">
-        <v>45288.54612149305</v>
+        <v>45138.4290727199</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mohamed.ElYamani1@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>45525.34441952546</v>
+          <t>Mahmoud.Farghel@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>004AD87E-8B2F-EE11-B8F0-6045BD8BD59A</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" s="1" t="n">
+        <v>45138.4290727199</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Mahmoud</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Farghel</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Mahmoud Farghel</t>
+        </is>
+      </c>
+      <c r="N35" s="1" t="n">
+        <v>46021.29896215278</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>FE49D87E-8B2F-EE11-B8F0-6045BD8BD59A</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Mahmoud.Farghel@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>62D70A47-82A5-EE11-8923-6045BD9E3927</t>
+          <t>9253FDC6-1A5E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B36" s="1" t="n">
-        <v>45288.54801292824</v>
+        <v>45523.46139667824</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mohamed.ElYamanii@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>45525.34416612268</v>
+          <t>Nermeen.Abdullah@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>9453FDC6-1A5E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" s="1" t="n">
+        <v>45523.46139667824</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Nermeen</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Mohamed Atia Abdullah</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Nermeen Mohamed Atia Abdullah</t>
+        </is>
+      </c>
+      <c r="N36" s="1" t="n">
+        <v>46213.3745087963</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="R36" s="1" t="n">
+        <v>45987.7844665162</v>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>9253FDC6-1A5E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Nermeen.Abdullah@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>55959A13-49AA-EE11-8923-6045BD9E3927</t>
+          <t>EC0A6DF4-345E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B37" s="1" t="n">
-        <v>45294.62666273148</v>
+        <v>45523.59156357639</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ola.abdelsabour@andalusiagroup.net</t>
+          <t>Eslam.Fawzy@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D37" s="1" t="n">
-        <v>45494.34981458334</v>
-      </c>
+        <v>45523.60411346065</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ED0A6DF4-345E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" s="1" t="n">
+        <v>45523.59156357639</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Eslam</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Fawzy</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Eslam Fawzy</t>
+        </is>
+      </c>
+      <c r="N37" s="1" t="n">
+        <v>45523.60411346065</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>EC0A6DF4-345E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>9253FDC6-1A5E-EF11-991A-6045BD9E3927</t>
+          <t>CFE14581-365E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B38" s="1" t="n">
-        <v>45523.46139667824</v>
+        <v>45523.59917399305</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Nermeen.Abdullah@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>Randa.AbdElMagid@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>45704.22445586805</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>D0E14581-365E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" s="1" t="n">
+        <v>45523.59917399305</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Randa</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>AbdElMagid</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Randa AbdElMagid</t>
+        </is>
+      </c>
+      <c r="N38" s="1" t="n">
+        <v>46218.57022642361</v>
+      </c>
+      <c r="O38" t="n">
+        <v>10</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R38" s="1" t="n">
+        <v>46218.39008711805</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>CFE14581-365E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Randa.AbdElMagid@Andalusiagroup.net</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>EC0A6DF4-345E-EF11-991A-6045BD9E3927</t>
+          <t>197A42A5-365E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>45523.59156357639</v>
+        <v>45523.59990065972</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eslam.Fawzy@Andalusiagroup.net</t>
+          <t>Nourhan.Elbana@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D39" s="1" t="n">
-        <v>45523.60411346065</v>
-      </c>
+        <v>45538.38317994213</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1A7A42A5-365E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" s="1" t="n">
+        <v>45523.59990065972</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Nourhan</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Elbana</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Nourhan Elbana</t>
+        </is>
+      </c>
+      <c r="N39" s="1" t="n">
+        <v>45538.38317994213</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R39" s="1" t="n">
+        <v>45535.55003287037</v>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>197A42A5-365E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CFE14581-365E-EF11-991A-6045BD9E3927</t>
+          <t>11151617-375E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B40" s="1" t="n">
-        <v>45523.59917399305</v>
+        <v>45523.60210625</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Randa.AbdElMagid@Andalusiagroup.net</t>
+          <t>Maha.Gamal@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D40" s="1" t="n">
-        <v>45704.22445586805</v>
+        <v>45723.25396666666</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>13151617-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" s="1" t="n">
+        <v>45523.60210625</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Maha</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Gamal</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Maha Gamal</t>
+        </is>
+      </c>
+      <c r="N40" s="1" t="n">
+        <v>46217.54598295139</v>
+      </c>
+      <c r="O40" t="n">
+        <v>10</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R40" s="1" t="n">
+        <v>46217.45874649306</v>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>11151617-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Maha.Gamal@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>197A42A5-365E-EF11-991A-6045BD9E3927</t>
+          <t>288FFC40-375E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B41" s="1" t="n">
-        <v>45523.59990065972</v>
+        <v>45523.60290783565</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Nourhan.Elbana@Andalusiagroup.net</t>
+          <t>Mahmoud.Mourad@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D41" s="1" t="n">
-        <v>45538.38317994213</v>
+        <v>45524.86951878472</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>298FFC40-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" s="1" t="n">
+        <v>45523.60290783565</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mahmoud </t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Gayad</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Mahmoud  Gayad</t>
+        </is>
+      </c>
+      <c r="N41" s="1" t="n">
+        <v>46218.84488506945</v>
+      </c>
+      <c r="O41" t="n">
+        <v>10</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R41" s="1" t="n">
+        <v>46218.84486623843</v>
+      </c>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>288FFC40-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Mahmoud.Gayad@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>11151617-375E-EF11-991A-6045BD9E3927</t>
+          <t>A5C40965-375E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B42" s="1" t="n">
-        <v>45523.60210625</v>
+        <v>45523.60366825231</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Maha.Gamal@Andalusiagroup.net</t>
+          <t>Sabry-Ahmed@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D42" s="1" t="n">
-        <v>45723.25396666666</v>
+        <v>45730.46087600695</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>A6C40965-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" s="1" t="n">
+        <v>45523.60366825231</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Rania</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Rania Mohamed</t>
+        </is>
+      </c>
+      <c r="N42" s="1" t="n">
+        <v>46218.47383464121</v>
+      </c>
+      <c r="O42" t="n">
+        <v>10</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R42" s="1" t="n">
+        <v>46218.4594037037</v>
+      </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>A5C40965-375E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Rania-Mohamed@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>288FFC40-375E-EF11-991A-6045BD9E3927</t>
+          <t>1171F26C-D65E-EF11-991A-6045BD9E3927</t>
         </is>
       </c>
       <c r="B43" s="1" t="n">
-        <v>45523.60290783565</v>
+        <v>45524.39422164352</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mahmoud.Mourad@Andalusiagroup.net</t>
+          <t>Ahmed-AboElGheit@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D43" s="1" t="n">
-        <v>45524.86951878472</v>
+        <v>45706.5892261574</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1271F26C-D65E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" s="1" t="n">
+        <v>45524.39422164352</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Ahmed</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Atef</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Ahmed Atef</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="n">
+        <v>46218.52092596065</v>
+      </c>
+      <c r="O43" t="n">
+        <v>10</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R43" s="1" t="n">
+        <v>46216.70722407407</v>
+      </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>1171F26C-D65E-EF11-991A-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Sayed.Saber@Andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>A5C40965-375E-EF11-991A-6045BD9E3927</t>
+          <t>62D70A47-82A5-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B44" s="1" t="n">
-        <v>45523.60366825231</v>
+        <v>45288.54801292824</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sabry-Ahmed@Andalusiagroup.net</t>
+          <t>Mohamed.ElYamanii@Andalusiagroup.net</t>
         </is>
       </c>
       <c r="D44" s="1" t="n">
-        <v>45730.46087600695</v>
-      </c>
+        <v>45525.34416612268</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>63D70A47-82A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" s="1" t="n">
+        <v>45288.54801292824</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Mohamed</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Magdy ElYamani Ali</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Mohamed Magdy ElYamani Ali</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="n">
+        <v>45322.69774236111</v>
+      </c>
+      <c r="O44" t="n">
+        <v>900</v>
+      </c>
+      <c r="P44" t="n">
+        <v>900</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R44" s="1" t="n">
+        <v>45296.52402033565</v>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>62D70A47-82A5-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1171F26C-D65E-EF11-991A-6045BD9E3927</t>
+          <t>55959A13-49AA-EE11-8923-6045BD9E3927</t>
         </is>
       </c>
       <c r="B45" s="1" t="n">
-        <v>45524.39422164352</v>
+        <v>45294.62666273148</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ahmed-AboElGheit@Andalusiagroup.net</t>
+          <t>ola.abdelsabour@andalusiagroup.net</t>
         </is>
       </c>
       <c r="D45" s="1" t="n">
-        <v>45706.5892261574</v>
-      </c>
+        <v>45494.34981458334</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>56959A13-49AA-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" s="1" t="n">
+        <v>45294.62666273148</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Ola</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>AbdelSabour</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Ola AbdelSabour</t>
+        </is>
+      </c>
+      <c r="N45" s="1" t="n">
+        <v>45494.34981458334</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>55959A13-49AA-EE11-8923-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>B278C7C1-D469-EF11-BDFD-6045BD9E3927</t>
+          <t>3FD1188C-817C-EE11-8923-000D3AACCC78</t>
         </is>
       </c>
       <c r="B46" s="1" t="n">
-        <v>45538.38429707176</v>
+        <v>45236.36845876157</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mona-Hassan@Andalusiagroup.net</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="n">
-        <v>45801.51275</v>
+          <t>Yosra.Hamed@Andalusiagroup.net</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>40D1188C-817C-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" s="1" t="n">
+        <v>45236.36845876157</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Eslam</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Saqr</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Eslam Saqr</t>
+        </is>
+      </c>
+      <c r="N46" s="1" t="n">
+        <v>46218.81709690972</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>3FD1188C-817C-EE11-8923-000D3AACCC78</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Eslam.ElSalam@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1252,6 +3908,65 @@
       </c>
       <c r="D47" s="1" t="n">
         <v>45323.37390825232</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>A00632F9-DFC0-EE11-BE9E-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" s="1" t="n">
+        <v>45323.37356357639</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Aya</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Mansour</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Aya Mansour</t>
+        </is>
+      </c>
+      <c r="N47" s="1" t="n">
+        <v>46218.50061859954</v>
+      </c>
+      <c r="O47" t="n">
+        <v>10</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="R47" s="1" t="n">
+        <v>46218.50060049768</v>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>9F0632F9-DFC0-EE11-BE9E-6045BD9E3927</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>aya.mansour@andalusiagroup.net</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>